<commit_message>
:white_circle: Dev v4.1.1: CH4 - Radar Plot
</commit_message>
<xml_diff>
--- a/02_Codigo/04_BattBankDesign/01_codes/02_Pnom025/01_Diseño_banco_batt_025.xlsx
+++ b/02_Codigo/04_BattBankDesign/01_codes/02_Pnom025/01_Diseño_banco_batt_025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dell PC\Desktop\Tesis Magister\02_Codigo\04_BattBankDesign\01_codes\02_Pnom025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F5D20DA-9777-41CE-8CA4-53EC5EDA7BCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4B21A29-4C11-4C2D-A20B-9B858C01AB31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-4695" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-4695" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1m_25%" sheetId="11" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="NMC" sheetId="5" r:id="rId4"/>
     <sheet name="LFP" sheetId="4" r:id="rId5"/>
     <sheet name="LTO" sheetId="6" r:id="rId6"/>
-    <sheet name="Radar_Plot_comparation" sheetId="14" r:id="rId7"/>
+    <sheet name="Radar_Plot" sheetId="14" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -992,7 +992,7 @@
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="105">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1132,23 +1132,41 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="7" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1162,30 +1180,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="7" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="5" xfId="2" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="43" fontId="7" fillId="0" borderId="5" xfId="2" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares" xfId="2" builtinId="3"/>
@@ -2623,7 +2617,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$D$14</c:f>
+              <c:f>Radar_Plot!$D$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2644,7 +2638,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$C$15:$C$19</c:f>
+              <c:f>Radar_Plot!$C$15:$C$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -2667,7 +2661,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$D$15:$D$19</c:f>
+              <c:f>Radar_Plot!$D$15:$D$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -2700,7 +2694,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$E$14</c:f>
+              <c:f>Radar_Plot!$E$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2721,7 +2715,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$C$15:$C$19</c:f>
+              <c:f>Radar_Plot!$C$15:$C$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -2744,7 +2738,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$E$15:$E$19</c:f>
+              <c:f>Radar_Plot!$E$15:$E$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -2777,7 +2771,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$F$14</c:f>
+              <c:f>Radar_Plot!$F$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2798,7 +2792,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$C$15:$C$19</c:f>
+              <c:f>Radar_Plot!$C$15:$C$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -2821,7 +2815,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$F$15:$F$19</c:f>
+              <c:f>Radar_Plot!$F$15:$F$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -2854,7 +2848,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$G$14</c:f>
+              <c:f>Radar_Plot!$G$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2875,7 +2869,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$C$15:$C$19</c:f>
+              <c:f>Radar_Plot!$C$15:$C$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -2898,7 +2892,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$G$15:$G$19</c:f>
+              <c:f>Radar_Plot!$G$15:$G$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3175,7 +3169,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AJ$14</c:f>
+              <c:f>Radar_Plot!$AJ$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3210,7 +3204,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AI$15:$AI$19</c:f>
+              <c:f>Radar_Plot!$AI$15:$AI$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3233,7 +3227,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$AJ$15:$AJ$19</c:f>
+              <c:f>Radar_Plot!$AJ$15:$AJ$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3266,7 +3260,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AK$14</c:f>
+              <c:f>Radar_Plot!$AK$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3301,7 +3295,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AI$15:$AI$19</c:f>
+              <c:f>Radar_Plot!$AI$15:$AI$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3324,7 +3318,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$AK$15:$AK$19</c:f>
+              <c:f>Radar_Plot!$AK$15:$AK$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3357,7 +3351,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AL$14</c:f>
+              <c:f>Radar_Plot!$AL$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3392,7 +3386,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AI$15:$AI$19</c:f>
+              <c:f>Radar_Plot!$AI$15:$AI$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3415,7 +3409,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$AL$15:$AL$19</c:f>
+              <c:f>Radar_Plot!$AL$15:$AL$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3699,7 +3693,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AB$14</c:f>
+              <c:f>Radar_Plot!$AB$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3734,7 +3728,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AA$15:$AA$19</c:f>
+              <c:f>Radar_Plot!$AA$15:$AA$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3757,7 +3751,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$AB$15:$AB$19</c:f>
+              <c:f>Radar_Plot!$AB$15:$AB$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3790,7 +3784,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AC$14</c:f>
+              <c:f>Radar_Plot!$AC$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3825,7 +3819,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AA$15:$AA$19</c:f>
+              <c:f>Radar_Plot!$AA$15:$AA$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3848,7 +3842,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$AC$15:$AC$19</c:f>
+              <c:f>Radar_Plot!$AC$15:$AC$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3881,7 +3875,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AD$14</c:f>
+              <c:f>Radar_Plot!$AD$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3916,7 +3910,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AA$15:$AA$19</c:f>
+              <c:f>Radar_Plot!$AA$15:$AA$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3939,7 +3933,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$AD$15:$AD$19</c:f>
+              <c:f>Radar_Plot!$AD$15:$AD$19</c:f>
               <c:numCache>
                 <c:formatCode>0</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3972,7 +3966,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AE$14</c:f>
+              <c:f>Radar_Plot!$AE$14</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4007,7 +4001,7 @@
           </c:marker>
           <c:cat>
             <c:strRef>
-              <c:f>Radar_Plot_comparation!$AA$15:$AA$19</c:f>
+              <c:f>Radar_Plot!$AA$15:$AA$19</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -4030,7 +4024,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Radar_Plot_comparation!$AE$15:$AE$19</c:f>
+              <c:f>Radar_Plot!$AE$15:$AE$19</c:f>
               <c:numCache>
                 <c:formatCode>0.00</c:formatCode>
                 <c:ptCount val="5"/>
@@ -5848,12 +5842,12 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:13" ht="18.75">
-      <c r="C5" s="81" t="s">
+      <c r="C5" s="92" t="s">
         <v>118</v>
       </c>
-      <c r="D5" s="81"/>
-      <c r="E5" s="81"/>
-      <c r="F5" s="81"/>
+      <c r="D5" s="92"/>
+      <c r="E5" s="92"/>
+      <c r="F5" s="92"/>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" s="37" t="s">
@@ -7798,13 +7792,13 @@
       <c r="J3" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="L3" s="84" t="s">
+      <c r="L3" s="93" t="s">
         <v>77</v>
       </c>
-      <c r="M3" s="82"/>
-      <c r="N3" s="82"/>
-      <c r="O3" s="82"/>
-      <c r="P3" s="82"/>
+      <c r="M3" s="94"/>
+      <c r="N3" s="94"/>
+      <c r="O3" s="94"/>
+      <c r="P3" s="94"/>
     </row>
     <row r="4" spans="3:16">
       <c r="C4" s="1" t="s">
@@ -9743,13 +9737,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:24" ht="15.75">
-      <c r="T2" s="84" t="s">
+      <c r="T2" s="93" t="s">
         <v>26</v>
       </c>
-      <c r="U2" s="82"/>
-      <c r="V2" s="82"/>
-      <c r="W2" s="82"/>
-      <c r="X2" s="82"/>
+      <c r="U2" s="94"/>
+      <c r="V2" s="94"/>
+      <c r="W2" s="94"/>
+      <c r="X2" s="94"/>
     </row>
     <row r="3" spans="3:24">
       <c r="C3" s="4" t="s">
@@ -10019,10 +10013,10 @@
       <c r="L11" s="1">
         <v>1920</v>
       </c>
-      <c r="O11" s="85" t="s">
+      <c r="O11" s="95" t="s">
         <v>50</v>
       </c>
-      <c r="P11" s="82"/>
+      <c r="P11" s="94"/>
     </row>
     <row r="12" spans="3:24">
       <c r="C12" s="1" t="s">
@@ -10186,10 +10180,10 @@
       <c r="L20" s="76">
         <v>750</v>
       </c>
-      <c r="O20" s="83" t="s">
+      <c r="O20" s="96" t="s">
         <v>63</v>
       </c>
-      <c r="P20" s="82"/>
+      <c r="P20" s="94"/>
     </row>
     <row r="21" spans="3:16" ht="15.75" customHeight="1">
       <c r="C21" s="1" t="s">
@@ -10298,10 +10292,10 @@
         <f>L23*L22</f>
         <v>38400</v>
       </c>
-      <c r="O24" s="86" t="s">
+      <c r="O24" s="97" t="s">
         <v>67</v>
       </c>
-      <c r="P24" s="82"/>
+      <c r="P24" s="94"/>
     </row>
     <row r="25" spans="3:16" ht="15.75" customHeight="1">
       <c r="C25" s="75" t="s">
@@ -10400,10 +10394,10 @@
         <f>L27*L26</f>
         <v>8250</v>
       </c>
-      <c r="O28" s="87" t="s">
+      <c r="O28" s="98" t="s">
         <v>114</v>
       </c>
-      <c r="P28" s="87"/>
+      <c r="P28" s="98"/>
     </row>
     <row r="29" spans="3:16" ht="15.75" customHeight="1">
       <c r="C29" s="9" t="s">
@@ -11868,11 +11862,11 @@
   </cols>
   <sheetData>
     <row r="2" spans="3:24" ht="15.75">
-      <c r="T2" s="84"/>
-      <c r="U2" s="82"/>
-      <c r="V2" s="82"/>
-      <c r="W2" s="82"/>
-      <c r="X2" s="82"/>
+      <c r="T2" s="93"/>
+      <c r="U2" s="94"/>
+      <c r="V2" s="94"/>
+      <c r="W2" s="94"/>
+      <c r="X2" s="94"/>
     </row>
     <row r="3" spans="3:24">
       <c r="C3" s="4" t="s">
@@ -12311,7 +12305,7 @@
       <c r="C27" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D27" s="99">
+      <c r="D27">
         <f>0.15</f>
         <v>0.15</v>
       </c>
@@ -13852,40 +13846,40 @@
   </cols>
   <sheetData>
     <row r="3" spans="3:38">
-      <c r="C3" s="88" t="s">
+      <c r="C3" s="100" t="s">
         <v>77</v>
       </c>
-      <c r="D3" s="89"/>
-      <c r="E3" s="89"/>
-      <c r="F3" s="89"/>
-      <c r="G3" s="90"/>
-      <c r="K3" s="88" t="s">
+      <c r="D3" s="101"/>
+      <c r="E3" s="101"/>
+      <c r="F3" s="101"/>
+      <c r="G3" s="102"/>
+      <c r="K3" s="100" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="91"/>
-      <c r="M3" s="91"/>
-      <c r="N3" s="91"/>
-      <c r="O3" s="92"/>
-      <c r="S3" s="88" t="s">
+      <c r="L3" s="103"/>
+      <c r="M3" s="103"/>
+      <c r="N3" s="103"/>
+      <c r="O3" s="104"/>
+      <c r="S3" s="100" t="s">
         <v>88</v>
       </c>
-      <c r="T3" s="91"/>
-      <c r="U3" s="91"/>
-      <c r="V3" s="91"/>
-      <c r="W3" s="92"/>
-      <c r="AA3" s="88" t="s">
+      <c r="T3" s="103"/>
+      <c r="U3" s="103"/>
+      <c r="V3" s="103"/>
+      <c r="W3" s="104"/>
+      <c r="AA3" s="100" t="s">
         <v>104</v>
       </c>
-      <c r="AB3" s="91"/>
-      <c r="AC3" s="91"/>
-      <c r="AD3" s="91"/>
-      <c r="AE3" s="92"/>
-      <c r="AI3" s="103" t="s">
+      <c r="AB3" s="103"/>
+      <c r="AC3" s="103"/>
+      <c r="AD3" s="103"/>
+      <c r="AE3" s="104"/>
+      <c r="AI3" s="99" t="s">
         <v>104</v>
       </c>
-      <c r="AJ3" s="103"/>
-      <c r="AK3" s="103"/>
-      <c r="AL3" s="103"/>
+      <c r="AJ3" s="99"/>
+      <c r="AK3" s="99"/>
+      <c r="AL3" s="99"/>
     </row>
     <row r="4" spans="3:38">
       <c r="C4" s="30"/>
@@ -13941,14 +13935,14 @@
         <v>82</v>
       </c>
       <c r="AG4" s="1"/>
-      <c r="AI4" s="104"/>
-      <c r="AJ4" s="104" t="s">
+      <c r="AI4" s="87"/>
+      <c r="AJ4" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="AK4" s="104" t="s">
+      <c r="AK4" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="AL4" s="104" t="s">
+      <c r="AL4" s="87" t="s">
         <v>82</v>
       </c>
     </row>
@@ -13962,7 +13956,7 @@
       <c r="E5" s="33">
         <v>1000</v>
       </c>
-      <c r="F5" s="93">
+      <c r="F5" s="81">
         <v>2000</v>
       </c>
       <c r="G5" s="34">
@@ -13978,7 +13972,7 @@
       <c r="M5" s="30">
         <v>2000</v>
       </c>
-      <c r="N5" s="96">
+      <c r="N5" s="83">
         <v>4000</v>
       </c>
       <c r="O5" s="30">
@@ -13988,7 +13982,7 @@
       <c r="S5" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="T5" s="97">
+      <c r="T5" s="84">
         <v>20000</v>
       </c>
       <c r="U5" s="34">
@@ -14012,7 +14006,7 @@
         <f>O5</f>
         <v>2500</v>
       </c>
-      <c r="AD5" s="97">
+      <c r="AD5" s="84">
         <f>W5</f>
         <v>13333.333333333334</v>
       </c>
@@ -14021,16 +14015,16 @@
         <v>5722.2222222222226</v>
       </c>
       <c r="AG5" s="1"/>
-      <c r="AI5" s="104" t="s">
+      <c r="AI5" s="87" t="s">
         <v>36</v>
       </c>
-      <c r="AJ5" s="104">
+      <c r="AJ5" s="87">
         <v>1333</v>
       </c>
-      <c r="AK5" s="107">
+      <c r="AK5" s="90">
         <v>2500</v>
       </c>
-      <c r="AL5" s="104">
+      <c r="AL5" s="87">
         <f>SUM(AJ5:AK5)/2</f>
         <v>1916.5</v>
       </c>
@@ -14039,7 +14033,7 @@
       <c r="C6" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="D6" s="93">
+      <c r="D6" s="81">
         <f>NMC!D29</f>
         <v>52542</v>
       </c>
@@ -14058,7 +14052,7 @@
       <c r="K6" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="L6" s="96">
+      <c r="L6" s="83">
         <f>LFP!D29</f>
         <v>64959</v>
       </c>
@@ -14081,7 +14075,7 @@
         <f>LTO!D29</f>
         <v>17500143</v>
       </c>
-      <c r="U6" s="97">
+      <c r="U6" s="84">
         <f>LTO!H29</f>
         <v>187500146</v>
       </c>
@@ -14104,7 +14098,7 @@
         <f t="shared" ref="AC6:AC9" si="4">O6</f>
         <v>26037.333333333332</v>
       </c>
-      <c r="AD6" s="97">
+      <c r="AD6" s="84">
         <f t="shared" ref="AD6:AD9" si="5">W6</f>
         <v>68916797.666666672</v>
       </c>
@@ -14113,16 +14107,16 @@
         <v>22990371.666666668</v>
       </c>
       <c r="AG6" s="1"/>
-      <c r="AI6" s="104" t="s">
+      <c r="AI6" s="87" t="s">
         <v>84</v>
       </c>
-      <c r="AJ6" s="107">
+      <c r="AJ6" s="90">
         <v>28280</v>
       </c>
-      <c r="AK6" s="105">
+      <c r="AK6" s="88">
         <v>26037.333333333332</v>
       </c>
-      <c r="AL6" s="105">
+      <c r="AL6" s="88">
         <f t="shared" ref="AL6:AL9" si="7">SUM(AJ6:AK6)/2</f>
         <v>27158.666666666664</v>
       </c>
@@ -14131,15 +14125,15 @@
       <c r="C7" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="D7" s="93">
+      <c r="D7" s="81">
         <f>NMC!D32</f>
         <v>42033.600000000006</v>
       </c>
-      <c r="E7" s="94">
+      <c r="E7" s="33">
         <f>NMC!G32</f>
         <v>36779.4</v>
       </c>
-      <c r="F7" s="94">
+      <c r="F7" s="33">
         <f>NMC!J32</f>
         <v>7096.32</v>
       </c>
@@ -14150,7 +14144,7 @@
       <c r="K7" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="L7" s="97">
+      <c r="L7" s="84">
         <f>LFP!D32</f>
         <v>64959</v>
       </c>
@@ -14173,7 +14167,7 @@
         <f>LTO!D32</f>
         <v>1575012.8699999999</v>
       </c>
-      <c r="U7" s="97">
+      <c r="U7" s="84">
         <f>LTO!H32</f>
         <v>225000.17519999997</v>
       </c>
@@ -14196,7 +14190,7 @@
         <f t="shared" si="4"/>
         <v>62914.299999999996</v>
       </c>
-      <c r="AD7" s="97">
+      <c r="AD7" s="84">
         <f t="shared" si="5"/>
         <v>626839.27639999997</v>
       </c>
@@ -14205,16 +14199,16 @@
         <v>239463.3388</v>
       </c>
       <c r="AG7" s="1"/>
-      <c r="AI7" s="104" t="s">
+      <c r="AI7" s="87" t="s">
         <v>85</v>
       </c>
-      <c r="AJ7" s="105">
+      <c r="AJ7" s="88">
         <v>28636.440000000002</v>
       </c>
-      <c r="AK7" s="108">
+      <c r="AK7" s="91">
         <v>62914.299999999996</v>
       </c>
-      <c r="AL7" s="105">
+      <c r="AL7" s="88">
         <f t="shared" si="7"/>
         <v>45775.369999999995</v>
       </c>
@@ -14223,15 +14217,15 @@
       <c r="C8" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="D8" s="94">
+      <c r="D8" s="33">
         <f>NMC!D34</f>
         <v>25.74558</v>
       </c>
-      <c r="E8" s="94">
+      <c r="E8" s="33">
         <f>NMC!G34</f>
         <v>19.738278000000001</v>
       </c>
-      <c r="F8" s="93">
+      <c r="F8" s="81">
         <f>NMC!J34</f>
         <v>28.108819200000003</v>
       </c>
@@ -14242,7 +14236,7 @@
       <c r="K8" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="L8" s="98">
+      <c r="L8" s="85">
         <f>LFP!D34</f>
         <v>59.045132639999999</v>
       </c>
@@ -14261,7 +14255,7 @@
       <c r="S8" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="T8" s="97">
+      <c r="T8" s="84">
         <f>LTO!D34</f>
         <v>3436.1450428481785</v>
       </c>
@@ -14288,7 +14282,7 @@
         <f t="shared" si="4"/>
         <v>51.074260822000006</v>
       </c>
-      <c r="AD8" s="97">
+      <c r="AD8" s="84">
         <f t="shared" si="5"/>
         <v>1299.7598630819245</v>
       </c>
@@ -14297,16 +14291,16 @@
         <v>458.45500543464158</v>
       </c>
       <c r="AG8" s="1"/>
-      <c r="AI8" s="104" t="s">
+      <c r="AI8" s="87" t="s">
         <v>57</v>
       </c>
-      <c r="AJ8" s="105">
+      <c r="AJ8" s="88">
         <v>24.530892399999999</v>
       </c>
-      <c r="AK8" s="108">
+      <c r="AK8" s="91">
         <v>51.074260822000006</v>
       </c>
-      <c r="AL8" s="105">
+      <c r="AL8" s="88">
         <f t="shared" si="7"/>
         <v>37.802576611000006</v>
       </c>
@@ -14315,15 +14309,15 @@
       <c r="C9" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="94">
+      <c r="D9" s="33">
         <f>NMC!D50</f>
         <v>3127.5</v>
       </c>
-      <c r="E9" s="93">
+      <c r="E9" s="81">
         <f>NMC!G50</f>
         <v>6255</v>
       </c>
-      <c r="F9" s="94">
+      <c r="F9" s="33">
         <f>NMC!J50</f>
         <v>5376</v>
       </c>
@@ -14334,7 +14328,7 @@
       <c r="K9" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="L9" s="97">
+      <c r="L9" s="84">
         <f>LFP!D50</f>
         <v>12386.25</v>
       </c>
@@ -14353,7 +14347,7 @@
       <c r="S9" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="T9" s="97">
+      <c r="T9" s="84">
         <f>LTO!D50</f>
         <v>6289.9875000000002</v>
       </c>
@@ -14376,11 +14370,11 @@
         <f t="shared" si="3"/>
         <v>4919.5</v>
       </c>
-      <c r="AC9" s="97">
+      <c r="AC9" s="84">
         <f t="shared" si="4"/>
         <v>8278.75</v>
       </c>
-      <c r="AD9" s="102">
+      <c r="AD9" s="34">
         <f t="shared" si="5"/>
         <v>5151.9859999999999</v>
       </c>
@@ -14388,55 +14382,55 @@
         <f t="shared" si="6"/>
         <v>6116.7453333333333</v>
       </c>
-      <c r="AI9" s="104" t="s">
+      <c r="AI9" s="87" t="s">
         <v>42</v>
       </c>
-      <c r="AJ9" s="105">
+      <c r="AJ9" s="88">
         <v>4919.5</v>
       </c>
-      <c r="AK9" s="108">
+      <c r="AK9" s="91">
         <v>8278.75</v>
       </c>
-      <c r="AL9" s="105">
+      <c r="AL9" s="88">
         <f t="shared" si="7"/>
         <v>6599.125</v>
       </c>
     </row>
     <row r="13" spans="3:38">
-      <c r="C13" s="88" t="s">
+      <c r="C13" s="100" t="s">
         <v>105</v>
       </c>
-      <c r="D13" s="91"/>
-      <c r="E13" s="91"/>
-      <c r="F13" s="91"/>
-      <c r="G13" s="92"/>
-      <c r="K13" s="88" t="s">
+      <c r="D13" s="103"/>
+      <c r="E13" s="103"/>
+      <c r="F13" s="103"/>
+      <c r="G13" s="104"/>
+      <c r="K13" s="100" t="s">
         <v>107</v>
       </c>
-      <c r="L13" s="91"/>
-      <c r="M13" s="91"/>
-      <c r="N13" s="91"/>
-      <c r="O13" s="92"/>
-      <c r="S13" s="88" t="s">
+      <c r="L13" s="103"/>
+      <c r="M13" s="103"/>
+      <c r="N13" s="103"/>
+      <c r="O13" s="104"/>
+      <c r="S13" s="100" t="s">
         <v>106</v>
       </c>
-      <c r="T13" s="91"/>
-      <c r="U13" s="91"/>
-      <c r="V13" s="91"/>
-      <c r="W13" s="92"/>
-      <c r="AA13" s="88" t="s">
+      <c r="T13" s="103"/>
+      <c r="U13" s="103"/>
+      <c r="V13" s="103"/>
+      <c r="W13" s="104"/>
+      <c r="AA13" s="100" t="s">
         <v>104</v>
       </c>
-      <c r="AB13" s="91"/>
-      <c r="AC13" s="91"/>
-      <c r="AD13" s="91"/>
-      <c r="AE13" s="92"/>
-      <c r="AI13" s="103" t="s">
+      <c r="AB13" s="103"/>
+      <c r="AC13" s="103"/>
+      <c r="AD13" s="103"/>
+      <c r="AE13" s="104"/>
+      <c r="AI13" s="99" t="s">
         <v>104</v>
       </c>
-      <c r="AJ13" s="103"/>
-      <c r="AK13" s="103"/>
-      <c r="AL13" s="103"/>
+      <c r="AJ13" s="99"/>
+      <c r="AK13" s="99"/>
+      <c r="AL13" s="99"/>
     </row>
     <row r="14" spans="3:38">
       <c r="C14" s="30"/>
@@ -14491,14 +14485,14 @@
       <c r="AE14" s="31" t="s">
         <v>82</v>
       </c>
-      <c r="AI14" s="104"/>
-      <c r="AJ14" s="104" t="s">
+      <c r="AI14" s="87"/>
+      <c r="AJ14" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="AK14" s="104" t="s">
+      <c r="AK14" s="87" t="s">
         <v>38</v>
       </c>
-      <c r="AL14" s="104" t="s">
+      <c r="AL14" s="87" t="s">
         <v>82</v>
       </c>
     </row>
@@ -14514,7 +14508,7 @@
         <f t="shared" ref="E15:G15" si="8">E5/$F$5</f>
         <v>0.5</v>
       </c>
-      <c r="F15" s="95">
+      <c r="F15" s="82">
         <f t="shared" si="8"/>
         <v>1</v>
       </c>
@@ -14533,7 +14527,7 @@
         <f t="shared" ref="M15:N15" si="9">M5/$N$5</f>
         <v>0.5</v>
       </c>
-      <c r="N15" s="97">
+      <c r="N15" s="84">
         <f t="shared" si="9"/>
         <v>1</v>
       </c>
@@ -14544,7 +14538,7 @@
       <c r="S15" s="32" t="s">
         <v>36</v>
       </c>
-      <c r="T15" s="97">
+      <c r="T15" s="84">
         <f>20000/20000</f>
         <v>1</v>
       </c>
@@ -14568,10 +14562,10 @@
         <v>9.9999999999999992E-2</v>
       </c>
       <c r="AC15" s="35">
-        <f t="shared" ref="AC15:AE15" si="11">AC5/$AD$5</f>
+        <f t="shared" ref="AC15:AD15" si="11">AC5/$AD$5</f>
         <v>0.1875</v>
       </c>
-      <c r="AD15" s="97">
+      <c r="AD15" s="84">
         <f t="shared" si="11"/>
         <v>1</v>
       </c>
@@ -14579,15 +14573,15 @@
       <c r="AI15" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="AJ15" s="106">
+      <c r="AJ15" s="89">
         <f>AJ5/$AK$5</f>
         <v>0.53320000000000001</v>
       </c>
-      <c r="AK15" s="108">
+      <c r="AK15" s="91">
         <f t="shared" ref="AK15:AL15" si="12">AK5/$AK$5</f>
         <v>1</v>
       </c>
-      <c r="AL15" s="106">
+      <c r="AL15" s="89">
         <f t="shared" si="12"/>
         <v>0.76659999999999995</v>
       </c>
@@ -14596,7 +14590,7 @@
       <c r="C16" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="D16" s="95">
+      <c r="D16" s="82">
         <f>D6/$D$6</f>
         <v>1</v>
       </c>
@@ -14615,7 +14609,7 @@
       <c r="K16" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="L16" s="96">
+      <c r="L16" s="83">
         <f>L6/$L$6</f>
         <v>1</v>
       </c>
@@ -14638,7 +14632,7 @@
         <f>139612/1491644</f>
         <v>9.3596059113300489E-2</v>
       </c>
-      <c r="U16" s="97">
+      <c r="U16" s="84">
         <f>1491644/1491644</f>
         <v>1</v>
       </c>
@@ -14658,10 +14652,10 @@
         <v>4.103498850422983E-4</v>
       </c>
       <c r="AC16" s="35">
-        <f t="shared" ref="AC16:AE16" si="15">AC6/$AD$6</f>
+        <f t="shared" ref="AC16:AD16" si="15">AC6/$AD$6</f>
         <v>3.778082298494107E-4</v>
       </c>
-      <c r="AD16" s="97">
+      <c r="AD16" s="84">
         <f t="shared" si="15"/>
         <v>1</v>
       </c>
@@ -14669,15 +14663,15 @@
       <c r="AI16" s="30" t="s">
         <v>84</v>
       </c>
-      <c r="AJ16" s="107">
+      <c r="AJ16" s="90">
         <f>AJ6/$AJ$6</f>
         <v>1</v>
       </c>
-      <c r="AK16" s="106">
+      <c r="AK16" s="89">
         <f t="shared" ref="AK16:AL16" si="16">AK6/$AJ$6</f>
         <v>0.92069778406412062</v>
       </c>
-      <c r="AL16" s="106">
+      <c r="AL16" s="89">
         <f t="shared" si="16"/>
         <v>0.96034889203206031</v>
       </c>
@@ -14686,7 +14680,7 @@
       <c r="C17" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="D17" s="95">
+      <c r="D17" s="82">
         <f>D7/$D$7</f>
         <v>1</v>
       </c>
@@ -14705,7 +14699,7 @@
       <c r="K17" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="L17" s="97">
+      <c r="L17" s="84">
         <f>L7/$L$7</f>
         <v>1</v>
       </c>
@@ -14728,7 +14722,7 @@
         <f>15.9261294244483/111.756922663701</f>
         <v>0.14250687156421815</v>
       </c>
-      <c r="U17" s="97">
+      <c r="U17" s="84">
         <f>111.756922663701/111.756922663701</f>
         <v>1</v>
       </c>
@@ -14743,15 +14737,15 @@
       <c r="AA17" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="AB17" s="100">
+      <c r="AB17" s="86">
         <f>AB7/$AD$7</f>
         <v>4.5683863596521761E-2</v>
       </c>
-      <c r="AC17" s="101">
-        <f t="shared" ref="AC17:AE17" si="19">AC7/$AD$7</f>
+      <c r="AC17" s="86">
+        <f t="shared" ref="AC17:AD17" si="19">AC7/$AD$7</f>
         <v>0.10036751423957198</v>
       </c>
-      <c r="AD17" s="97">
+      <c r="AD17" s="84">
         <f t="shared" si="19"/>
         <v>1</v>
       </c>
@@ -14759,15 +14753,15 @@
       <c r="AI17" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="AJ17" s="106">
+      <c r="AJ17" s="89">
         <f>AJ7/$AK$7</f>
         <v>0.45516583670167204</v>
       </c>
-      <c r="AK17" s="108">
+      <c r="AK17" s="91">
         <f t="shared" ref="AK17:AL17" si="20">AK7/$AK$7</f>
         <v>1</v>
       </c>
-      <c r="AL17" s="106">
+      <c r="AL17" s="89">
         <f t="shared" si="20"/>
         <v>0.72758291835083599</v>
       </c>
@@ -14784,7 +14778,7 @@
         <f t="shared" ref="E18:G18" si="21">E8/$F$8</f>
         <v>0.70220943325858376</v>
       </c>
-      <c r="F18" s="95">
+      <c r="F18" s="82">
         <f t="shared" si="21"/>
         <v>1</v>
       </c>
@@ -14795,7 +14789,7 @@
       <c r="K18" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="L18" s="97">
+      <c r="L18" s="84">
         <f>L8/$L$8</f>
         <v>1</v>
       </c>
@@ -14814,7 +14808,7 @@
       <c r="S18" s="32" t="s">
         <v>43</v>
       </c>
-      <c r="T18" s="97">
+      <c r="T18" s="84">
         <f>T7/$T$7</f>
         <v>1</v>
       </c>
@@ -14838,10 +14832,10 @@
         <v>1.8873403539199612E-2</v>
       </c>
       <c r="AC18" s="35">
-        <f t="shared" ref="AC18:AE18" si="24">AC8/$AD$8</f>
+        <f t="shared" ref="AC18:AD18" si="24">AC8/$AD$8</f>
         <v>3.9295151568148376E-2</v>
       </c>
-      <c r="AD18" s="97">
+      <c r="AD18" s="84">
         <f t="shared" si="24"/>
         <v>1</v>
       </c>
@@ -14849,15 +14843,15 @@
       <c r="AI18" s="30" t="s">
         <v>57</v>
       </c>
-      <c r="AJ18" s="106">
+      <c r="AJ18" s="89">
         <f>AJ8/$AK$8</f>
         <v>0.480298530124462</v>
       </c>
-      <c r="AK18" s="108">
+      <c r="AK18" s="91">
         <f t="shared" ref="AK18:AL18" si="25">AK8/$AK$8</f>
         <v>1</v>
       </c>
-      <c r="AL18" s="106">
+      <c r="AL18" s="89">
         <f t="shared" si="25"/>
         <v>0.74014926506223111</v>
       </c>
@@ -14870,7 +14864,7 @@
         <f>D9/$E$9</f>
         <v>0.5</v>
       </c>
-      <c r="E19" s="95">
+      <c r="E19" s="82">
         <f t="shared" ref="E19:G19" si="26">E9/$E$9</f>
         <v>1</v>
       </c>
@@ -14885,7 +14879,7 @@
       <c r="K19" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="L19" s="96">
+      <c r="L19" s="83">
         <f>L9/$L$9</f>
         <v>1</v>
       </c>
@@ -14904,7 +14898,7 @@
       <c r="S19" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="T19" s="97">
+      <c r="T19" s="84">
         <f>T9/$T$9</f>
         <v>1</v>
       </c>
@@ -14927,8 +14921,8 @@
         <f>AB9/$AC$9</f>
         <v>0.59423222104786355</v>
       </c>
-      <c r="AC19" s="97">
-        <f t="shared" ref="AC19:AE19" si="29">AC9/$AC$9</f>
+      <c r="AC19" s="84">
+        <f t="shared" ref="AC19:AD19" si="29">AC9/$AC$9</f>
         <v>1</v>
       </c>
       <c r="AD19" s="35">
@@ -14939,15 +14933,15 @@
       <c r="AI19" s="30" t="s">
         <v>42</v>
       </c>
-      <c r="AJ19" s="106">
+      <c r="AJ19" s="89">
         <f>AJ9/$AK$9</f>
         <v>0.59423222104786355</v>
       </c>
-      <c r="AK19" s="108">
+      <c r="AK19" s="91">
         <f t="shared" ref="AK19:AL19" si="30">AK9/$AK$9</f>
         <v>1</v>
       </c>
-      <c r="AL19" s="106">
+      <c r="AL19" s="89">
         <f t="shared" si="30"/>
         <v>0.79711611052393172</v>
       </c>

</xml_diff>